<commit_message>
feat(reviews): añadir 1 valoración(es) de clientes (test alexa) vía n8n
</commit_message>
<xml_diff>
--- a/data/reviews-clients.xlsx
+++ b/data/reviews-clients.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -619,9 +619,29 @@
         <v>1a1697a45682b1eb</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>test alexa</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>El pedido llegó incompleto</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-10-23T16:01:15.000Z</v>
+      </c>
+      <c r="F12" t="str">
+        <v>1a1697ec896664d8</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(reviews): añadir 1 valoración(es) de clientes (María García) vía n8n
</commit_message>
<xml_diff>
--- a/data/reviews-clients.xlsx
+++ b/data/reviews-clients.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -639,9 +639,29 @@
         <v>1a1697ec896664d8</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>María García</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v>El pedido llegó tarde y el producto estaba dañado.</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2026-10-26T18:42:03.647Z</v>
+      </c>
+      <c r="F13" t="str">
+        <v>PRUEBA-001</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(reviews): añadir 1 valoración(es) de clientes (Ana pruebazdskj) vía n8n
</commit_message>
<xml_diff>
--- a/data/reviews-clients.xlsx
+++ b/data/reviews-clients.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -659,9 +659,29 @@
         <v>PRUEBA-001</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Ana pruebazdskj</v>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v>El pedido llegó tarde, con el envase roto y nadie avisó</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2026-10-26T18:54:34.000Z</v>
+      </c>
+      <c r="F14" t="str">
+        <v>1a179908643f6518</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F14"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>